<commit_message>
Team Capture as of 10/09/2026
</commit_message>
<xml_diff>
--- a/data/2026/cjsl/fall/brooklyn-premier-fc-14-13-regional.xlsx
+++ b/data/2026/cjsl/fall/brooklyn-premier-fc-14-13-regional.xlsx
@@ -78,7 +78,7 @@
     <col min="6" max="6" bestFit="1" customWidth="1" width="45.1"/>
     <col min="7" max="7" bestFit="1" customWidth="1" width="49.50000000000001"/>
     <col min="8" max="8" bestFit="1" customWidth="1" width="22.0"/>
-    <col min="9" max="9" bestFit="1" customWidth="1" width="11.0"/>
+    <col min="9" max="9" bestFit="1" customWidth="1" width="12.100000000000001"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -175,21 +175,21 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Sunday, September 27, 2026</t>
+          <t>Saturday, October 17, 2026</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>11:00 EDT</t>
+          <t>16:00 EDT</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn Premier F.C. 14/13 Regional</t>
+          <t>Soccer Fun for Kids / Brooklyn Patriots 2013-2014</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
@@ -199,12 +199,12 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>Chernomorets Black Sea 2014</t>
+          <t>Brooklyn Premier F.C. 14/13 Regional</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>KAISER PARK - KAISER PARK</t>
+          <t>Prospect Park, Parade Grounds Field 10A - Parade Grounds Field 10A</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -214,27 +214,27 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>Rained Out</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Saturday, October 17, 2026</t>
+          <t>Sunday, October 18, 2026</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>16:00 EDT</t>
+          <t>11:00 EDT</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Soccer Fun for Kids / Brooklyn Patriots 2013-2014</t>
+          <t>Brooklyn Premier F.C. 14/13 Regional</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
@@ -244,12 +244,12 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn Premier F.C. 14/13 Regional</t>
+          <t>Chernomorets Black Sea 2014</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>Prospect Park, Parade Grounds Field 10A - Parade Grounds Field 10A</t>
+          <t>KAISER PARK - KAISER PARK</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -259,7 +259,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Rescheduled</t>
         </is>
       </c>
     </row>

</xml_diff>